<commit_message>
began testing functions, edited functions, updated logic
</commit_message>
<xml_diff>
--- a/src/TestExcelSheet.xlsx
+++ b/src/TestExcelSheet.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Cassie\Documents\.vscode\personal projects\Carone Fitness\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Cassie\Documents\.vscode\personal projects\Carone Fitness\datasift-xl\src\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{31B65689-35C0-4439-9E5A-AA80C96EA84A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{52DA0BFA-3566-4B5A-83AC-974877BFC2E9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1900" yWindow="1900" windowWidth="14400" windowHeight="7270" activeTab="1" xr2:uid="{14B052A0-022B-4FBE-9E4C-795118B232C0}"/>
+    <workbookView xWindow="380" yWindow="380" windowWidth="14400" windowHeight="7270" xr2:uid="{14B052A0-022B-4FBE-9E4C-795118B232C0}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -19,7 +19,6 @@
     <sheet name="Some other dumb name" sheetId="3" r:id="rId4"/>
   </sheets>
   <calcPr calcId="191029"/>
-  <fileRecoveryPr repairLoad="1"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -40,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="379" uniqueCount="171">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="391" uniqueCount="181">
   <si>
     <t>Bool</t>
   </si>
@@ -557,6 +556,36 @@
   </si>
   <si>
     <t>Female Athlete Triad</t>
+  </si>
+  <si>
+    <t>1a</t>
+  </si>
+  <si>
+    <t>2a</t>
+  </si>
+  <si>
+    <t>3a</t>
+  </si>
+  <si>
+    <t>5a</t>
+  </si>
+  <si>
+    <t>6a</t>
+  </si>
+  <si>
+    <t>7a</t>
+  </si>
+  <si>
+    <t>8a</t>
+  </si>
+  <si>
+    <t>9a</t>
+  </si>
+  <si>
+    <t>10a</t>
+  </si>
+  <si>
+    <t>11a</t>
   </si>
 </sst>
 </file>
@@ -616,7 +645,6 @@
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="10" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
@@ -634,6 +662,7 @@
     <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
@@ -997,8 +1026,8 @@
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A2">
-        <v>1</v>
+      <c r="A2" t="s">
+        <v>171</v>
       </c>
       <c r="B2" t="s">
         <v>5</v>
@@ -1017,9 +1046,8 @@
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A3">
-        <f>A2 +1</f>
-        <v>2</v>
+      <c r="A3" t="s">
+        <v>172</v>
       </c>
       <c r="B3" t="s">
         <v>6</v>
@@ -1038,9 +1066,8 @@
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A4">
-        <f t="shared" ref="A4:A12" si="0">A3 +1</f>
-        <v>3</v>
+      <c r="A4" t="s">
+        <v>173</v>
       </c>
       <c r="B4" t="s">
         <v>7</v>
@@ -1059,10 +1086,6 @@
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A5">
-        <f t="shared" si="0"/>
-        <v>4</v>
-      </c>
       <c r="B5" t="s">
         <v>8</v>
       </c>
@@ -1080,9 +1103,8 @@
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A6">
-        <f t="shared" si="0"/>
-        <v>5</v>
+      <c r="A6" t="s">
+        <v>174</v>
       </c>
       <c r="B6" t="s">
         <v>9</v>
@@ -1101,9 +1123,8 @@
       </c>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A7">
-        <f t="shared" si="0"/>
-        <v>6</v>
+      <c r="A7" t="s">
+        <v>175</v>
       </c>
       <c r="B7" t="s">
         <v>10</v>
@@ -1122,9 +1143,8 @@
       </c>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A8">
-        <f t="shared" si="0"/>
-        <v>7</v>
+      <c r="A8" t="s">
+        <v>176</v>
       </c>
       <c r="B8" t="s">
         <v>11</v>
@@ -1143,9 +1163,8 @@
       </c>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A9">
-        <f t="shared" si="0"/>
-        <v>8</v>
+      <c r="A9" t="s">
+        <v>177</v>
       </c>
       <c r="B9" t="s">
         <v>12</v>
@@ -1164,9 +1183,8 @@
       </c>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A10">
-        <f t="shared" si="0"/>
-        <v>9</v>
+      <c r="A10" t="s">
+        <v>178</v>
       </c>
       <c r="B10" t="s">
         <v>13</v>
@@ -1185,9 +1203,8 @@
       </c>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A11">
-        <f t="shared" si="0"/>
-        <v>10</v>
+      <c r="A11" t="s">
+        <v>179</v>
       </c>
       <c r="B11" t="s">
         <v>14</v>
@@ -1206,9 +1223,8 @@
       </c>
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A12">
-        <f t="shared" si="0"/>
-        <v>11</v>
+      <c r="A12" t="s">
+        <v>180</v>
       </c>
       <c r="B12" t="s">
         <v>15</v>
@@ -1240,71 +1256,71 @@
       <c r="A1" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="B1" s="4" t="s">
+      <c r="B1" s="11" t="s">
         <v>24</v>
       </c>
-      <c r="C1" s="4"/>
-      <c r="D1" s="4"/>
-      <c r="E1" s="4"/>
-      <c r="F1" s="4"/>
-      <c r="G1" s="4"/>
-      <c r="H1" s="4"/>
-      <c r="I1" s="4"/>
-      <c r="J1" s="4"/>
+      <c r="C1" s="11"/>
+      <c r="D1" s="11"/>
+      <c r="E1" s="11"/>
+      <c r="F1" s="11"/>
+      <c r="G1" s="11"/>
+      <c r="H1" s="11"/>
+      <c r="I1" s="11"/>
+      <c r="J1" s="11"/>
     </row>
     <row r="2" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A2" s="3" t="s">
         <v>25</v>
       </c>
-      <c r="B2" s="4" t="s">
+      <c r="B2" s="11" t="s">
         <v>26</v>
       </c>
-      <c r="C2" s="4"/>
-      <c r="D2" s="4"/>
-      <c r="E2" s="4"/>
-      <c r="F2" s="4"/>
-      <c r="G2" s="4"/>
-      <c r="H2" s="4"/>
-      <c r="I2" s="4"/>
-      <c r="J2" s="4"/>
+      <c r="C2" s="11"/>
+      <c r="D2" s="11"/>
+      <c r="E2" s="11"/>
+      <c r="F2" s="11"/>
+      <c r="G2" s="11"/>
+      <c r="H2" s="11"/>
+      <c r="I2" s="11"/>
+      <c r="J2" s="11"/>
     </row>
     <row r="4" spans="1:10" ht="58" x14ac:dyDescent="0.35">
-      <c r="A4" s="5" t="s">
+      <c r="A4" s="4" t="s">
         <v>27</v>
       </c>
-      <c r="B4" s="5" t="s">
+      <c r="B4" s="4" t="s">
         <v>28</v>
       </c>
-      <c r="C4" s="6" t="s">
+      <c r="C4" s="5" t="s">
         <v>29</v>
       </c>
-      <c r="D4" s="6" t="s">
+      <c r="D4" s="5" t="s">
         <v>30</v>
       </c>
-      <c r="E4" s="5" t="s">
+      <c r="E4" s="4" t="s">
         <v>31</v>
       </c>
-      <c r="F4" s="6" t="s">
+      <c r="F4" s="5" t="s">
         <v>32</v>
       </c>
-      <c r="G4" s="6" t="s">
+      <c r="G4" s="5" t="s">
         <v>33</v>
       </c>
-      <c r="H4" s="7" t="s">
+      <c r="H4" s="6" t="s">
         <v>34</v>
       </c>
     </row>
     <row r="5" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A5" s="8" t="s">
+      <c r="A5" s="7" t="s">
         <v>35</v>
       </c>
-      <c r="B5" s="8"/>
-      <c r="C5" s="8"/>
-      <c r="D5" s="8"/>
-      <c r="E5" s="8"/>
-      <c r="F5" s="8"/>
-      <c r="G5" s="8"/>
-      <c r="H5" s="8"/>
+      <c r="B5" s="7"/>
+      <c r="C5" s="7"/>
+      <c r="D5" s="7"/>
+      <c r="E5" s="7"/>
+      <c r="F5" s="7"/>
+      <c r="G5" s="7"/>
+      <c r="H5" s="7"/>
     </row>
     <row r="6" spans="1:10" x14ac:dyDescent="0.35">
       <c r="B6" t="s">
@@ -1335,28 +1351,28 @@
       </c>
     </row>
     <row r="8" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A8" s="6" t="s">
+      <c r="A8" s="5" t="s">
         <v>40</v>
       </c>
-      <c r="B8" s="6"/>
-      <c r="C8" s="6"/>
-      <c r="D8" s="6"/>
-      <c r="E8" s="6"/>
-      <c r="F8" s="6"/>
-      <c r="G8" s="6"/>
-      <c r="H8" s="6"/>
+      <c r="B8" s="5"/>
+      <c r="C8" s="5"/>
+      <c r="D8" s="5"/>
+      <c r="E8" s="5"/>
+      <c r="F8" s="5"/>
+      <c r="G8" s="5"/>
+      <c r="H8" s="5"/>
     </row>
     <row r="9" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A9" s="8" t="s">
+      <c r="A9" s="7" t="s">
         <v>41</v>
       </c>
-      <c r="B9" s="8"/>
-      <c r="C9" s="8"/>
-      <c r="D9" s="8"/>
-      <c r="E9" s="8"/>
-      <c r="F9" s="8"/>
-      <c r="G9" s="8"/>
-      <c r="H9" s="8"/>
+      <c r="B9" s="7"/>
+      <c r="C9" s="7"/>
+      <c r="D9" s="7"/>
+      <c r="E9" s="7"/>
+      <c r="F9" s="7"/>
+      <c r="G9" s="7"/>
+      <c r="H9" s="7"/>
     </row>
     <row r="10" spans="1:10" x14ac:dyDescent="0.35">
       <c r="B10" t="s">
@@ -1376,162 +1392,162 @@
       </c>
     </row>
     <row r="11" spans="1:10" ht="43.5" x14ac:dyDescent="0.35">
-      <c r="A11" s="9"/>
-      <c r="B11" s="9" t="s">
+      <c r="A11" s="8"/>
+      <c r="B11" s="8" t="s">
         <v>43</v>
       </c>
-      <c r="C11" s="9" t="s">
-        <v>37</v>
-      </c>
-      <c r="D11" s="9"/>
-      <c r="E11" s="9">
+      <c r="C11" s="8" t="s">
+        <v>37</v>
+      </c>
+      <c r="D11" s="8"/>
+      <c r="E11" s="8">
         <v>10</v>
       </c>
-      <c r="F11" s="9" t="s">
-        <v>37</v>
-      </c>
-      <c r="G11" s="9"/>
-      <c r="H11" s="9" t="s">
+      <c r="F11" s="8" t="s">
+        <v>37</v>
+      </c>
+      <c r="G11" s="8"/>
+      <c r="H11" s="8" t="s">
         <v>44</v>
       </c>
     </row>
     <row r="12" spans="1:10" ht="43.5" x14ac:dyDescent="0.35">
-      <c r="A12" s="9"/>
-      <c r="B12" s="9" t="s">
+      <c r="A12" s="8"/>
+      <c r="B12" s="8" t="s">
         <v>45</v>
       </c>
-      <c r="C12" s="9" t="s">
+      <c r="C12" s="8" t="s">
         <v>46</v>
       </c>
-      <c r="D12" s="9"/>
-      <c r="E12" s="9">
+      <c r="D12" s="8"/>
+      <c r="E12" s="8">
         <v>4</v>
       </c>
-      <c r="F12" s="9" t="s">
+      <c r="F12" s="8" t="s">
         <v>46</v>
       </c>
-      <c r="G12" s="9"/>
-      <c r="H12" s="9" t="s">
+      <c r="G12" s="8"/>
+      <c r="H12" s="8" t="s">
         <v>47</v>
       </c>
     </row>
     <row r="13" spans="1:10" ht="29" x14ac:dyDescent="0.35">
-      <c r="A13" s="9"/>
-      <c r="B13" s="9" t="s">
+      <c r="A13" s="8"/>
+      <c r="B13" s="8" t="s">
         <v>48</v>
       </c>
-      <c r="C13" s="9" t="s">
-        <v>37</v>
-      </c>
-      <c r="D13" s="9"/>
-      <c r="E13" s="9">
+      <c r="C13" s="8" t="s">
+        <v>37</v>
+      </c>
+      <c r="D13" s="8"/>
+      <c r="E13" s="8">
         <v>10</v>
       </c>
-      <c r="F13" s="9" t="s">
-        <v>37</v>
-      </c>
-      <c r="G13" s="9"/>
-      <c r="H13" s="9" t="s">
+      <c r="F13" s="8" t="s">
+        <v>37</v>
+      </c>
+      <c r="G13" s="8"/>
+      <c r="H13" s="8" t="s">
         <v>44</v>
       </c>
     </row>
     <row r="14" spans="1:10" ht="43.5" x14ac:dyDescent="0.35">
-      <c r="A14" s="7" t="s">
+      <c r="A14" s="6" t="s">
         <v>49</v>
       </c>
-      <c r="B14" s="7"/>
-      <c r="C14" s="7"/>
-      <c r="D14" s="7"/>
-      <c r="E14" s="7">
+      <c r="B14" s="6"/>
+      <c r="C14" s="6"/>
+      <c r="D14" s="6"/>
+      <c r="E14" s="6">
         <v>7</v>
       </c>
-      <c r="F14" s="7" t="s">
-        <v>37</v>
-      </c>
-      <c r="G14" s="7"/>
-      <c r="H14" s="7" t="s">
+      <c r="F14" s="6" t="s">
+        <v>37</v>
+      </c>
+      <c r="G14" s="6"/>
+      <c r="H14" s="6" t="s">
         <v>44</v>
       </c>
     </row>
     <row r="15" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A15" s="8" t="s">
+      <c r="A15" s="7" t="s">
         <v>50</v>
       </c>
-      <c r="B15" s="8"/>
-      <c r="C15" s="8"/>
-      <c r="D15" s="8"/>
-      <c r="E15" s="8"/>
-      <c r="F15" s="8"/>
-      <c r="G15" s="8"/>
-      <c r="H15" s="8"/>
+      <c r="B15" s="7"/>
+      <c r="C15" s="7"/>
+      <c r="D15" s="7"/>
+      <c r="E15" s="7"/>
+      <c r="F15" s="7"/>
+      <c r="G15" s="7"/>
+      <c r="H15" s="7"/>
     </row>
     <row r="16" spans="1:10" ht="87" x14ac:dyDescent="0.35">
-      <c r="A16" s="9"/>
-      <c r="B16" s="9" t="s">
+      <c r="A16" s="8"/>
+      <c r="B16" s="8" t="s">
         <v>51</v>
       </c>
-      <c r="C16" s="9" t="s">
+      <c r="C16" s="8" t="s">
         <v>52</v>
       </c>
-      <c r="D16" s="9" t="s">
+      <c r="D16" s="8" t="s">
         <v>53</v>
       </c>
-      <c r="E16" s="9">
+      <c r="E16" s="8">
         <v>7</v>
       </c>
-      <c r="F16" s="9" t="s">
+      <c r="F16" s="8" t="s">
         <v>54</v>
       </c>
-      <c r="G16" s="9" t="s">
+      <c r="G16" s="8" t="s">
         <v>55</v>
       </c>
-      <c r="H16" s="9"/>
+      <c r="H16" s="8"/>
     </row>
     <row r="17" spans="1:8" ht="101.5" x14ac:dyDescent="0.35">
-      <c r="A17" s="9"/>
-      <c r="B17" s="9" t="s">
+      <c r="A17" s="8"/>
+      <c r="B17" s="8" t="s">
         <v>56</v>
       </c>
-      <c r="C17" s="9" t="s">
+      <c r="C17" s="8" t="s">
         <v>57</v>
       </c>
-      <c r="D17" s="9" t="s">
+      <c r="D17" s="8" t="s">
         <v>58</v>
       </c>
-      <c r="E17" s="9">
+      <c r="E17" s="8">
         <v>7</v>
       </c>
-      <c r="F17" s="9" t="s">
-        <v>37</v>
-      </c>
-      <c r="G17" s="9" t="s">
+      <c r="F17" s="8" t="s">
+        <v>37</v>
+      </c>
+      <c r="G17" s="8" t="s">
         <v>59</v>
       </c>
-      <c r="H17" s="9" t="s">
+      <c r="H17" s="8" t="s">
         <v>60</v>
       </c>
     </row>
     <row r="18" spans="1:8" ht="203" x14ac:dyDescent="0.35">
-      <c r="A18" s="9"/>
-      <c r="B18" s="9" t="s">
+      <c r="A18" s="8"/>
+      <c r="B18" s="8" t="s">
         <v>61</v>
       </c>
-      <c r="C18" s="9" t="s">
+      <c r="C18" s="8" t="s">
         <v>57</v>
       </c>
-      <c r="D18" s="9" t="s">
+      <c r="D18" s="8" t="s">
         <v>62</v>
       </c>
-      <c r="E18" s="9">
+      <c r="E18" s="8">
         <v>6</v>
       </c>
-      <c r="F18" s="9" t="s">
-        <v>37</v>
-      </c>
-      <c r="G18" s="9" t="s">
+      <c r="F18" s="8" t="s">
+        <v>37</v>
+      </c>
+      <c r="G18" s="8" t="s">
         <v>55</v>
       </c>
-      <c r="H18" s="9" t="s">
+      <c r="H18" s="8" t="s">
         <v>63</v>
       </c>
     </row>
@@ -1547,322 +1563,322 @@
       </c>
     </row>
     <row r="20" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A20" s="8" t="s">
+      <c r="A20" s="7" t="s">
         <v>65</v>
       </c>
-      <c r="B20" s="8"/>
-      <c r="C20" s="8"/>
-      <c r="D20" s="8"/>
-      <c r="E20" s="8"/>
-      <c r="F20" s="8"/>
-      <c r="G20" s="8"/>
-      <c r="H20" s="8"/>
+      <c r="B20" s="7"/>
+      <c r="C20" s="7"/>
+      <c r="D20" s="7"/>
+      <c r="E20" s="7"/>
+      <c r="F20" s="7"/>
+      <c r="G20" s="7"/>
+      <c r="H20" s="7"/>
     </row>
     <row r="21" spans="1:8" ht="29" x14ac:dyDescent="0.35">
-      <c r="A21" s="9"/>
-      <c r="B21" s="9" t="s">
+      <c r="A21" s="8"/>
+      <c r="B21" s="8" t="s">
         <v>66</v>
       </c>
-      <c r="C21" s="9" t="s">
-        <v>37</v>
-      </c>
-      <c r="D21" s="9"/>
-      <c r="E21" s="9">
+      <c r="C21" s="8" t="s">
+        <v>37</v>
+      </c>
+      <c r="D21" s="8"/>
+      <c r="E21" s="8">
         <v>8</v>
       </c>
-      <c r="F21" s="9" t="s">
-        <v>37</v>
-      </c>
-      <c r="G21" s="9" t="s">
+      <c r="F21" s="8" t="s">
+        <v>37</v>
+      </c>
+      <c r="G21" s="8" t="s">
         <v>67</v>
       </c>
-      <c r="H21" s="9" t="s">
+      <c r="H21" s="8" t="s">
         <v>68</v>
       </c>
     </row>
     <row r="22" spans="1:8" ht="145" x14ac:dyDescent="0.35">
-      <c r="A22" s="9"/>
-      <c r="B22" s="9" t="s">
+      <c r="A22" s="8"/>
+      <c r="B22" s="8" t="s">
         <v>69</v>
       </c>
-      <c r="C22" s="9" t="s">
+      <c r="C22" s="8" t="s">
         <v>70</v>
       </c>
-      <c r="D22" s="9"/>
-      <c r="E22" s="9">
+      <c r="D22" s="8"/>
+      <c r="E22" s="8">
         <v>7</v>
       </c>
       <c r="F22" t="s">
         <v>37</v>
       </c>
-      <c r="G22" s="9" t="s">
+      <c r="G22" s="8" t="s">
         <v>71</v>
       </c>
-      <c r="H22" s="9" t="s">
+      <c r="H22" s="8" t="s">
         <v>72</v>
       </c>
     </row>
     <row r="23" spans="1:8" ht="43.5" x14ac:dyDescent="0.35">
-      <c r="A23" s="9"/>
-      <c r="B23" s="9" t="s">
+      <c r="A23" s="8"/>
+      <c r="B23" s="8" t="s">
         <v>73</v>
       </c>
-      <c r="C23" s="9" t="s">
+      <c r="C23" s="8" t="s">
         <v>46</v>
       </c>
-      <c r="D23" s="9"/>
-      <c r="E23" s="9">
+      <c r="D23" s="8"/>
+      <c r="E23" s="8">
         <v>1</v>
       </c>
       <c r="F23" t="s">
         <v>46</v>
       </c>
-      <c r="G23" s="9"/>
-      <c r="H23" s="9" t="s">
+      <c r="G23" s="8"/>
+      <c r="H23" s="8" t="s">
         <v>72</v>
       </c>
     </row>
     <row r="24" spans="1:8" ht="43.5" x14ac:dyDescent="0.35">
-      <c r="A24" s="9"/>
-      <c r="B24" s="9" t="s">
+      <c r="A24" s="8"/>
+      <c r="B24" s="8" t="s">
         <v>74</v>
       </c>
-      <c r="C24" s="9" t="s">
-        <v>37</v>
-      </c>
-      <c r="D24" s="9" t="s">
+      <c r="C24" s="8" t="s">
+        <v>37</v>
+      </c>
+      <c r="D24" s="8" t="s">
         <v>75</v>
       </c>
-      <c r="E24" s="9">
+      <c r="E24" s="8">
         <v>9</v>
       </c>
       <c r="F24" t="s">
         <v>37</v>
       </c>
-      <c r="G24" s="9"/>
-      <c r="H24" s="9" t="s">
+      <c r="G24" s="8"/>
+      <c r="H24" s="8" t="s">
         <v>76</v>
       </c>
     </row>
     <row r="25" spans="1:8" ht="87" x14ac:dyDescent="0.35">
-      <c r="A25" s="9"/>
-      <c r="B25" s="9" t="s">
+      <c r="A25" s="8"/>
+      <c r="B25" s="8" t="s">
         <v>77</v>
       </c>
-      <c r="C25" s="9" t="s">
-        <v>37</v>
-      </c>
-      <c r="D25" s="9"/>
-      <c r="E25" s="9">
+      <c r="C25" s="8" t="s">
+        <v>37</v>
+      </c>
+      <c r="D25" s="8"/>
+      <c r="E25" s="8">
         <v>7</v>
       </c>
-      <c r="G25" s="9" t="s">
+      <c r="G25" s="8" t="s">
         <v>78</v>
       </c>
-      <c r="H25" s="9" t="s">
+      <c r="H25" s="8" t="s">
         <v>72</v>
       </c>
     </row>
     <row r="26" spans="1:8" ht="29" x14ac:dyDescent="0.35">
-      <c r="A26" s="9"/>
-      <c r="B26" s="9" t="s">
+      <c r="A26" s="8"/>
+      <c r="B26" s="8" t="s">
         <v>48</v>
       </c>
-      <c r="C26" s="9" t="s">
+      <c r="C26" s="8" t="s">
         <v>70</v>
       </c>
-      <c r="D26" s="9"/>
-      <c r="E26" s="9">
+      <c r="D26" s="8"/>
+      <c r="E26" s="8">
         <v>3</v>
       </c>
-      <c r="F26" s="9" t="s">
+      <c r="F26" s="8" t="s">
         <v>70</v>
       </c>
-      <c r="G26" s="9"/>
-      <c r="H26" s="9" t="s">
+      <c r="G26" s="8"/>
+      <c r="H26" s="8" t="s">
         <v>72</v>
       </c>
     </row>
     <row r="27" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A27" s="8" t="s">
+      <c r="A27" s="7" t="s">
         <v>79</v>
       </c>
-      <c r="B27" s="8"/>
-      <c r="C27" s="8"/>
-      <c r="D27" s="8"/>
-      <c r="E27" s="8"/>
-      <c r="F27" s="8"/>
-      <c r="G27" s="8"/>
-      <c r="H27" s="8"/>
+      <c r="B27" s="7"/>
+      <c r="C27" s="7"/>
+      <c r="D27" s="7"/>
+      <c r="E27" s="7"/>
+      <c r="F27" s="7"/>
+      <c r="G27" s="7"/>
+      <c r="H27" s="7"/>
     </row>
     <row r="28" spans="1:8" ht="29" x14ac:dyDescent="0.35">
-      <c r="A28" s="9"/>
-      <c r="B28" s="9" t="s">
+      <c r="A28" s="8"/>
+      <c r="B28" s="8" t="s">
         <v>80</v>
       </c>
-      <c r="C28" s="9" t="s">
-        <v>37</v>
-      </c>
-      <c r="D28" s="9"/>
-      <c r="E28" s="9">
+      <c r="C28" s="8" t="s">
+        <v>37</v>
+      </c>
+      <c r="D28" s="8"/>
+      <c r="E28" s="8">
         <v>6</v>
       </c>
       <c r="F28" t="s">
         <v>37</v>
       </c>
-      <c r="G28" s="9"/>
-      <c r="H28" s="9" t="s">
+      <c r="G28" s="8"/>
+      <c r="H28" s="8" t="s">
         <v>68</v>
       </c>
     </row>
     <row r="29" spans="1:8" ht="116" x14ac:dyDescent="0.35">
-      <c r="A29" s="9"/>
-      <c r="B29" s="9" t="s">
+      <c r="A29" s="8"/>
+      <c r="B29" s="8" t="s">
         <v>81</v>
       </c>
-      <c r="C29" s="9" t="s">
-        <v>37</v>
-      </c>
-      <c r="D29" s="9" t="s">
+      <c r="C29" s="8" t="s">
+        <v>37</v>
+      </c>
+      <c r="D29" s="8" t="s">
         <v>82</v>
       </c>
-      <c r="E29" s="9">
+      <c r="E29" s="8">
         <v>4</v>
       </c>
-      <c r="G29" s="9" t="s">
+      <c r="G29" s="8" t="s">
         <v>55</v>
       </c>
-      <c r="H29" s="9" t="s">
+      <c r="H29" s="8" t="s">
         <v>83</v>
       </c>
     </row>
     <row r="30" spans="1:8" ht="87" x14ac:dyDescent="0.35">
-      <c r="A30" s="9"/>
-      <c r="B30" s="9" t="s">
+      <c r="A30" s="8"/>
+      <c r="B30" s="8" t="s">
         <v>84</v>
       </c>
-      <c r="C30" s="9" t="s">
+      <c r="C30" s="8" t="s">
         <v>85</v>
       </c>
-      <c r="D30" s="9" t="s">
+      <c r="D30" s="8" t="s">
         <v>86</v>
       </c>
-      <c r="E30" s="9">
+      <c r="E30" s="8">
         <v>7</v>
       </c>
-      <c r="F30" s="9"/>
-      <c r="G30" s="9" t="s">
+      <c r="F30" s="8"/>
+      <c r="G30" s="8" t="s">
         <v>59</v>
       </c>
-      <c r="H30" s="9" t="s">
+      <c r="H30" s="8" t="s">
         <v>87</v>
       </c>
     </row>
     <row r="31" spans="1:8" ht="43.5" x14ac:dyDescent="0.35">
-      <c r="A31" s="9"/>
-      <c r="B31" s="9" t="s">
+      <c r="A31" s="8"/>
+      <c r="B31" s="8" t="s">
         <v>48</v>
       </c>
-      <c r="C31" s="9" t="s">
+      <c r="C31" s="8" t="s">
         <v>85</v>
       </c>
-      <c r="D31" s="9" t="s">
+      <c r="D31" s="8" t="s">
         <v>88</v>
       </c>
-      <c r="E31" s="9">
+      <c r="E31" s="8">
         <v>7</v>
       </c>
-      <c r="F31" s="9"/>
-      <c r="G31" s="9" t="s">
+      <c r="F31" s="8"/>
+      <c r="G31" s="8" t="s">
         <v>59</v>
       </c>
-      <c r="H31" s="9" t="s">
+      <c r="H31" s="8" t="s">
         <v>87</v>
       </c>
     </row>
     <row r="32" spans="1:8" ht="58" x14ac:dyDescent="0.35">
-      <c r="A32" s="7" t="s">
+      <c r="A32" s="6" t="s">
         <v>89</v>
       </c>
-      <c r="B32" s="7"/>
-      <c r="C32" s="7"/>
-      <c r="D32" s="7"/>
-      <c r="E32" s="7"/>
-      <c r="F32" s="7"/>
-      <c r="G32" s="7"/>
-      <c r="H32" s="7"/>
+      <c r="B32" s="6"/>
+      <c r="C32" s="6"/>
+      <c r="D32" s="6"/>
+      <c r="E32" s="6"/>
+      <c r="F32" s="6"/>
+      <c r="G32" s="6"/>
+      <c r="H32" s="6"/>
     </row>
     <row r="33" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A33" s="8" t="s">
+      <c r="A33" s="7" t="s">
         <v>90</v>
       </c>
-      <c r="B33" s="10"/>
-      <c r="C33" s="10"/>
-      <c r="D33" s="10"/>
-      <c r="E33" s="10"/>
-      <c r="F33" s="10"/>
-      <c r="G33" s="10"/>
-      <c r="H33" s="10"/>
+      <c r="B33" s="9"/>
+      <c r="C33" s="9"/>
+      <c r="D33" s="9"/>
+      <c r="E33" s="9"/>
+      <c r="F33" s="9"/>
+      <c r="G33" s="9"/>
+      <c r="H33" s="9"/>
     </row>
     <row r="34" spans="1:8" ht="116" x14ac:dyDescent="0.35">
-      <c r="A34" s="9"/>
-      <c r="B34" s="9" t="s">
+      <c r="A34" s="8"/>
+      <c r="B34" s="8" t="s">
         <v>91</v>
       </c>
-      <c r="C34" s="9" t="s">
-        <v>37</v>
-      </c>
-      <c r="D34" s="9"/>
-      <c r="E34" s="9">
+      <c r="C34" s="8" t="s">
+        <v>37</v>
+      </c>
+      <c r="D34" s="8"/>
+      <c r="E34" s="8">
         <v>15</v>
       </c>
-      <c r="F34" s="9" t="s">
-        <v>37</v>
-      </c>
-      <c r="G34" s="9" t="s">
+      <c r="F34" s="8" t="s">
+        <v>37</v>
+      </c>
+      <c r="G34" s="8" t="s">
         <v>92</v>
       </c>
-      <c r="H34" s="9" t="s">
+      <c r="H34" s="8" t="s">
         <v>83</v>
       </c>
     </row>
     <row r="35" spans="1:8" ht="29" x14ac:dyDescent="0.35">
-      <c r="A35" s="9"/>
-      <c r="B35" s="9" t="s">
+      <c r="A35" s="8"/>
+      <c r="B35" s="8" t="s">
         <v>93</v>
       </c>
-      <c r="C35" s="9" t="s">
-        <v>37</v>
-      </c>
-      <c r="D35" s="9"/>
-      <c r="E35" s="9">
+      <c r="C35" s="8" t="s">
+        <v>37</v>
+      </c>
+      <c r="D35" s="8"/>
+      <c r="E35" s="8">
         <v>1</v>
       </c>
-      <c r="F35" s="9" t="s">
-        <v>37</v>
-      </c>
-      <c r="G35" s="9"/>
-      <c r="H35" s="9" t="s">
+      <c r="F35" s="8" t="s">
+        <v>37</v>
+      </c>
+      <c r="G35" s="8"/>
+      <c r="H35" s="8" t="s">
         <v>83</v>
       </c>
     </row>
     <row r="36" spans="1:8" ht="58" x14ac:dyDescent="0.35">
-      <c r="A36" s="9"/>
-      <c r="B36" s="9" t="s">
+      <c r="A36" s="8"/>
+      <c r="B36" s="8" t="s">
         <v>94</v>
       </c>
-      <c r="C36" s="9" t="s">
-        <v>37</v>
-      </c>
-      <c r="D36" s="9"/>
-      <c r="E36" s="9">
+      <c r="C36" s="8" t="s">
+        <v>37</v>
+      </c>
+      <c r="D36" s="8"/>
+      <c r="E36" s="8">
         <v>2</v>
       </c>
-      <c r="F36" s="9" t="s">
-        <v>37</v>
-      </c>
-      <c r="G36" s="9"/>
-      <c r="H36" s="9" t="s">
+      <c r="F36" s="8" t="s">
+        <v>37</v>
+      </c>
+      <c r="G36" s="8"/>
+      <c r="H36" s="8" t="s">
         <v>83</v>
       </c>
     </row>
@@ -1870,16 +1886,16 @@
       <c r="B37" t="s">
         <v>95</v>
       </c>
-      <c r="C37" s="9" t="s">
-        <v>37</v>
-      </c>
-      <c r="E37" s="9">
+      <c r="C37" s="8" t="s">
+        <v>37</v>
+      </c>
+      <c r="E37" s="8">
         <v>2</v>
       </c>
-      <c r="F37" s="9" t="s">
-        <v>37</v>
-      </c>
-      <c r="H37" s="9" t="s">
+      <c r="F37" s="8" t="s">
+        <v>37</v>
+      </c>
+      <c r="H37" s="8" t="s">
         <v>83</v>
       </c>
     </row>
@@ -1887,167 +1903,167 @@
       <c r="B38" t="s">
         <v>48</v>
       </c>
-      <c r="C38" s="9" t="s">
-        <v>37</v>
-      </c>
-      <c r="F38" s="9"/>
-      <c r="H38" s="9" t="s">
+      <c r="C38" s="8" t="s">
+        <v>37</v>
+      </c>
+      <c r="F38" s="8"/>
+      <c r="H38" s="8" t="s">
         <v>83</v>
       </c>
     </row>
     <row r="39" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A39" s="8" t="s">
+      <c r="A39" s="7" t="s">
         <v>96</v>
       </c>
-      <c r="B39" s="8"/>
-      <c r="C39" s="8"/>
-      <c r="D39" s="8"/>
-      <c r="E39" s="8"/>
-      <c r="F39" s="8"/>
-      <c r="G39" s="8"/>
-      <c r="H39" s="8"/>
+      <c r="B39" s="7"/>
+      <c r="C39" s="7"/>
+      <c r="D39" s="7"/>
+      <c r="E39" s="7"/>
+      <c r="F39" s="7"/>
+      <c r="G39" s="7"/>
+      <c r="H39" s="7"/>
     </row>
     <row r="40" spans="1:8" ht="58" x14ac:dyDescent="0.35">
-      <c r="A40" s="9"/>
-      <c r="B40" s="9" t="s">
+      <c r="A40" s="8"/>
+      <c r="B40" s="8" t="s">
         <v>97</v>
       </c>
-      <c r="C40" s="9" t="s">
-        <v>37</v>
-      </c>
-      <c r="D40" s="9"/>
-      <c r="E40" s="9">
+      <c r="C40" s="8" t="s">
+        <v>37</v>
+      </c>
+      <c r="D40" s="8"/>
+      <c r="E40" s="8">
         <v>8</v>
       </c>
-      <c r="F40" s="9" t="s">
-        <v>37</v>
-      </c>
-      <c r="G40" s="9"/>
-      <c r="H40" s="9" t="s">
+      <c r="F40" s="8" t="s">
+        <v>37</v>
+      </c>
+      <c r="G40" s="8"/>
+      <c r="H40" s="8" t="s">
         <v>83</v>
       </c>
     </row>
     <row r="41" spans="1:8" ht="43.5" x14ac:dyDescent="0.35">
-      <c r="A41" s="9"/>
-      <c r="B41" s="9" t="s">
+      <c r="A41" s="8"/>
+      <c r="B41" s="8" t="s">
         <v>98</v>
       </c>
-      <c r="C41" s="9" t="s">
-        <v>37</v>
-      </c>
-      <c r="D41" s="9"/>
-      <c r="E41" s="9">
+      <c r="C41" s="8" t="s">
+        <v>37</v>
+      </c>
+      <c r="D41" s="8"/>
+      <c r="E41" s="8">
         <v>4</v>
       </c>
-      <c r="F41" s="9" t="s">
-        <v>37</v>
-      </c>
-      <c r="G41" s="9"/>
-      <c r="H41" s="9" t="s">
+      <c r="F41" s="8" t="s">
+        <v>37</v>
+      </c>
+      <c r="G41" s="8"/>
+      <c r="H41" s="8" t="s">
         <v>83</v>
       </c>
     </row>
     <row r="42" spans="1:8" ht="29" x14ac:dyDescent="0.35">
-      <c r="A42" s="9"/>
-      <c r="B42" s="9" t="s">
+      <c r="A42" s="8"/>
+      <c r="B42" s="8" t="s">
         <v>99</v>
       </c>
-      <c r="C42" s="9" t="s">
-        <v>37</v>
-      </c>
-      <c r="D42" s="9"/>
-      <c r="E42" s="9">
+      <c r="C42" s="8" t="s">
+        <v>37</v>
+      </c>
+      <c r="D42" s="8"/>
+      <c r="E42" s="8">
         <v>8</v>
       </c>
-      <c r="F42" s="9" t="s">
-        <v>37</v>
-      </c>
-      <c r="G42" s="9"/>
-      <c r="H42" s="9" t="s">
+      <c r="F42" s="8" t="s">
+        <v>37</v>
+      </c>
+      <c r="G42" s="8"/>
+      <c r="H42" s="8" t="s">
         <v>83</v>
       </c>
     </row>
     <row r="43" spans="1:8" ht="29" x14ac:dyDescent="0.35">
-      <c r="A43" s="9"/>
-      <c r="B43" s="9" t="s">
+      <c r="A43" s="8"/>
+      <c r="B43" s="8" t="s">
         <v>48</v>
       </c>
-      <c r="C43" s="9" t="s">
-        <v>37</v>
-      </c>
-      <c r="D43" s="9"/>
-      <c r="E43" s="9"/>
-      <c r="F43" s="9"/>
-      <c r="G43" s="9"/>
-      <c r="H43" s="9" t="s">
+      <c r="C43" s="8" t="s">
+        <v>37</v>
+      </c>
+      <c r="D43" s="8"/>
+      <c r="E43" s="8"/>
+      <c r="F43" s="8"/>
+      <c r="G43" s="8"/>
+      <c r="H43" s="8" t="s">
         <v>83</v>
       </c>
     </row>
     <row r="44" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A44" s="11" t="s">
+      <c r="A44" s="10" t="s">
         <v>100</v>
       </c>
-      <c r="B44" s="11"/>
-      <c r="C44" s="11"/>
-      <c r="D44" s="11"/>
-      <c r="E44" s="11"/>
-      <c r="F44" s="11"/>
-      <c r="G44" s="11"/>
-      <c r="H44" s="11"/>
+      <c r="B44" s="10"/>
+      <c r="C44" s="10"/>
+      <c r="D44" s="10"/>
+      <c r="E44" s="10"/>
+      <c r="F44" s="10"/>
+      <c r="G44" s="10"/>
+      <c r="H44" s="10"/>
     </row>
     <row r="45" spans="1:8" ht="43.5" x14ac:dyDescent="0.35">
-      <c r="A45" s="9"/>
-      <c r="B45" s="9" t="s">
+      <c r="A45" s="8"/>
+      <c r="B45" s="8" t="s">
         <v>101</v>
       </c>
-      <c r="C45" s="9" t="s">
-        <v>37</v>
-      </c>
-      <c r="D45" s="9"/>
-      <c r="E45" s="9">
+      <c r="C45" s="8" t="s">
+        <v>37</v>
+      </c>
+      <c r="D45" s="8"/>
+      <c r="E45" s="8">
         <v>11</v>
       </c>
-      <c r="F45" s="9" t="s">
-        <v>37</v>
-      </c>
-      <c r="G45" s="9"/>
-      <c r="H45" s="9" t="s">
+      <c r="F45" s="8" t="s">
+        <v>37</v>
+      </c>
+      <c r="G45" s="8"/>
+      <c r="H45" s="8" t="s">
         <v>83</v>
       </c>
     </row>
     <row r="46" spans="1:8" ht="43.5" x14ac:dyDescent="0.35">
-      <c r="A46" s="9"/>
-      <c r="B46" s="9" t="s">
+      <c r="A46" s="8"/>
+      <c r="B46" s="8" t="s">
         <v>102</v>
       </c>
-      <c r="C46" s="9" t="s">
-        <v>37</v>
-      </c>
-      <c r="D46" s="9"/>
-      <c r="E46" s="9">
+      <c r="C46" s="8" t="s">
+        <v>37</v>
+      </c>
+      <c r="D46" s="8"/>
+      <c r="E46" s="8">
         <v>9</v>
       </c>
-      <c r="F46" s="9" t="s">
-        <v>37</v>
-      </c>
-      <c r="G46" s="9"/>
-      <c r="H46" s="9" t="s">
+      <c r="F46" s="8" t="s">
+        <v>37</v>
+      </c>
+      <c r="G46" s="8"/>
+      <c r="H46" s="8" t="s">
         <v>83</v>
       </c>
     </row>
     <row r="47" spans="1:8" ht="29" x14ac:dyDescent="0.35">
-      <c r="A47" s="9"/>
-      <c r="B47" s="9" t="s">
+      <c r="A47" s="8"/>
+      <c r="B47" s="8" t="s">
         <v>48</v>
       </c>
-      <c r="C47" s="9" t="s">
-        <v>37</v>
-      </c>
-      <c r="D47" s="9"/>
-      <c r="E47" s="9"/>
-      <c r="F47" s="9"/>
-      <c r="G47" s="9"/>
-      <c r="H47" s="9" t="s">
+      <c r="C47" s="8" t="s">
+        <v>37</v>
+      </c>
+      <c r="D47" s="8"/>
+      <c r="E47" s="8"/>
+      <c r="F47" s="8"/>
+      <c r="G47" s="8"/>
+      <c r="H47" s="8" t="s">
         <v>83</v>
       </c>
     </row>
@@ -2064,198 +2080,198 @@
       <c r="H48" s="12"/>
     </row>
     <row r="49" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A49" s="11" t="s">
+      <c r="A49" s="10" t="s">
         <v>104</v>
       </c>
-      <c r="B49" s="11"/>
-      <c r="C49" s="11"/>
-      <c r="D49" s="11"/>
-      <c r="E49" s="11"/>
-      <c r="F49" s="11"/>
-      <c r="G49" s="11"/>
-      <c r="H49" s="11"/>
+      <c r="B49" s="10"/>
+      <c r="C49" s="10"/>
+      <c r="D49" s="10"/>
+      <c r="E49" s="10"/>
+      <c r="F49" s="10"/>
+      <c r="G49" s="10"/>
+      <c r="H49" s="10"/>
     </row>
     <row r="50" spans="1:8" ht="29" x14ac:dyDescent="0.35">
-      <c r="A50" s="9"/>
-      <c r="B50" s="9" t="s">
+      <c r="A50" s="8"/>
+      <c r="B50" s="8" t="s">
         <v>105</v>
       </c>
-      <c r="C50" s="9" t="s">
-        <v>37</v>
-      </c>
-      <c r="D50" s="9"/>
-      <c r="E50" s="9">
+      <c r="C50" s="8" t="s">
+        <v>37</v>
+      </c>
+      <c r="D50" s="8"/>
+      <c r="E50" s="8">
         <v>4</v>
       </c>
-      <c r="F50" s="9" t="s">
-        <v>37</v>
-      </c>
-      <c r="G50" s="9"/>
-      <c r="H50" s="9" t="s">
+      <c r="F50" s="8" t="s">
+        <v>37</v>
+      </c>
+      <c r="G50" s="8"/>
+      <c r="H50" s="8" t="s">
         <v>83</v>
       </c>
     </row>
     <row r="51" spans="1:8" ht="29" x14ac:dyDescent="0.35">
-      <c r="A51" s="9"/>
-      <c r="B51" s="9" t="s">
+      <c r="A51" s="8"/>
+      <c r="B51" s="8" t="s">
         <v>106</v>
       </c>
-      <c r="C51" s="9" t="s">
-        <v>37</v>
-      </c>
-      <c r="D51" s="9"/>
-      <c r="E51" s="9">
+      <c r="C51" s="8" t="s">
+        <v>37</v>
+      </c>
+      <c r="D51" s="8"/>
+      <c r="E51" s="8">
         <v>13</v>
       </c>
-      <c r="F51" s="9" t="s">
-        <v>37</v>
-      </c>
-      <c r="G51" s="9"/>
-      <c r="H51" s="9" t="s">
+      <c r="F51" s="8" t="s">
+        <v>37</v>
+      </c>
+      <c r="G51" s="8"/>
+      <c r="H51" s="8" t="s">
         <v>83</v>
       </c>
     </row>
     <row r="52" spans="1:8" ht="43.5" x14ac:dyDescent="0.35">
-      <c r="A52" s="9"/>
-      <c r="B52" s="9" t="s">
+      <c r="A52" s="8"/>
+      <c r="B52" s="8" t="s">
         <v>107</v>
       </c>
-      <c r="C52" s="9" t="s">
-        <v>37</v>
-      </c>
-      <c r="D52" s="9"/>
-      <c r="E52" s="9">
+      <c r="C52" s="8" t="s">
+        <v>37</v>
+      </c>
+      <c r="D52" s="8"/>
+      <c r="E52" s="8">
         <v>3</v>
       </c>
-      <c r="F52" s="9" t="s">
-        <v>37</v>
-      </c>
-      <c r="G52" s="9"/>
-      <c r="H52" s="9" t="s">
+      <c r="F52" s="8" t="s">
+        <v>37</v>
+      </c>
+      <c r="G52" s="8"/>
+      <c r="H52" s="8" t="s">
         <v>83</v>
       </c>
     </row>
     <row r="53" spans="1:8" ht="29" x14ac:dyDescent="0.35">
-      <c r="A53" s="9"/>
-      <c r="B53" s="9" t="s">
+      <c r="A53" s="8"/>
+      <c r="B53" s="8" t="s">
         <v>48</v>
       </c>
-      <c r="C53" s="9" t="s">
-        <v>37</v>
-      </c>
-      <c r="D53" s="9"/>
-      <c r="E53" s="9"/>
-      <c r="F53" s="9"/>
-      <c r="G53" s="9"/>
-      <c r="H53" s="9" t="s">
+      <c r="C53" s="8" t="s">
+        <v>37</v>
+      </c>
+      <c r="D53" s="8"/>
+      <c r="E53" s="8"/>
+      <c r="F53" s="8"/>
+      <c r="G53" s="8"/>
+      <c r="H53" s="8" t="s">
         <v>83</v>
       </c>
     </row>
     <row r="54" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A54" s="11" t="s">
+      <c r="A54" s="10" t="s">
         <v>108</v>
       </c>
-      <c r="B54" s="11"/>
-      <c r="C54" s="11"/>
-      <c r="D54" s="11"/>
-      <c r="E54" s="11"/>
-      <c r="F54" s="11"/>
-      <c r="G54" s="11"/>
-      <c r="H54" s="11"/>
+      <c r="B54" s="10"/>
+      <c r="C54" s="10"/>
+      <c r="D54" s="10"/>
+      <c r="E54" s="10"/>
+      <c r="F54" s="10"/>
+      <c r="G54" s="10"/>
+      <c r="H54" s="10"/>
     </row>
     <row r="55" spans="1:8" ht="29" x14ac:dyDescent="0.35">
-      <c r="A55" s="9"/>
-      <c r="B55" s="9" t="s">
+      <c r="A55" s="8"/>
+      <c r="B55" s="8" t="s">
         <v>109</v>
       </c>
-      <c r="C55" s="9" t="s">
-        <v>37</v>
-      </c>
-      <c r="D55" s="9"/>
-      <c r="E55" s="9">
+      <c r="C55" s="8" t="s">
+        <v>37</v>
+      </c>
+      <c r="D55" s="8"/>
+      <c r="E55" s="8">
         <v>3</v>
       </c>
-      <c r="F55" s="9" t="s">
-        <v>37</v>
-      </c>
-      <c r="G55" s="9"/>
-      <c r="H55" s="9" t="s">
+      <c r="F55" s="8" t="s">
+        <v>37</v>
+      </c>
+      <c r="G55" s="8"/>
+      <c r="H55" s="8" t="s">
         <v>110</v>
       </c>
     </row>
     <row r="56" spans="1:8" ht="43.5" x14ac:dyDescent="0.35">
-      <c r="A56" s="9"/>
-      <c r="B56" s="9" t="s">
+      <c r="A56" s="8"/>
+      <c r="B56" s="8" t="s">
         <v>111</v>
       </c>
-      <c r="C56" s="9" t="s">
-        <v>37</v>
-      </c>
-      <c r="D56" s="9"/>
-      <c r="E56" s="9">
+      <c r="C56" s="8" t="s">
+        <v>37</v>
+      </c>
+      <c r="D56" s="8"/>
+      <c r="E56" s="8">
         <v>4</v>
       </c>
-      <c r="F56" s="9" t="s">
-        <v>37</v>
-      </c>
-      <c r="G56" s="9"/>
-      <c r="H56" s="9" t="s">
+      <c r="F56" s="8" t="s">
+        <v>37</v>
+      </c>
+      <c r="G56" s="8"/>
+      <c r="H56" s="8" t="s">
         <v>110</v>
       </c>
     </row>
     <row r="57" spans="1:8" ht="43.5" x14ac:dyDescent="0.35">
-      <c r="A57" s="9"/>
-      <c r="B57" s="9" t="s">
+      <c r="A57" s="8"/>
+      <c r="B57" s="8" t="s">
         <v>112</v>
       </c>
-      <c r="C57" s="9" t="s">
-        <v>37</v>
-      </c>
-      <c r="D57" s="9"/>
-      <c r="E57" s="9">
+      <c r="C57" s="8" t="s">
+        <v>37</v>
+      </c>
+      <c r="D57" s="8"/>
+      <c r="E57" s="8">
         <v>4</v>
       </c>
-      <c r="F57" s="9" t="s">
-        <v>37</v>
-      </c>
-      <c r="G57" s="9"/>
-      <c r="H57" s="9" t="s">
+      <c r="F57" s="8" t="s">
+        <v>37</v>
+      </c>
+      <c r="G57" s="8"/>
+      <c r="H57" s="8" t="s">
         <v>110</v>
       </c>
     </row>
     <row r="58" spans="1:8" ht="43.5" x14ac:dyDescent="0.35">
-      <c r="A58" s="9"/>
-      <c r="B58" s="9" t="s">
+      <c r="A58" s="8"/>
+      <c r="B58" s="8" t="s">
         <v>113</v>
       </c>
-      <c r="C58" s="9" t="s">
-        <v>37</v>
-      </c>
-      <c r="D58" s="9"/>
-      <c r="E58" s="9">
+      <c r="C58" s="8" t="s">
+        <v>37</v>
+      </c>
+      <c r="D58" s="8"/>
+      <c r="E58" s="8">
         <v>9</v>
       </c>
-      <c r="F58" s="9" t="s">
-        <v>37</v>
-      </c>
-      <c r="G58" s="9"/>
-      <c r="H58" s="9" t="s">
+      <c r="F58" s="8" t="s">
+        <v>37</v>
+      </c>
+      <c r="G58" s="8"/>
+      <c r="H58" s="8" t="s">
         <v>110</v>
       </c>
     </row>
     <row r="59" spans="1:8" ht="29" x14ac:dyDescent="0.35">
-      <c r="A59" s="9"/>
-      <c r="B59" s="9" t="s">
+      <c r="A59" s="8"/>
+      <c r="B59" s="8" t="s">
         <v>48</v>
       </c>
-      <c r="C59" s="9" t="s">
-        <v>37</v>
-      </c>
-      <c r="D59" s="9"/>
-      <c r="E59" s="9"/>
-      <c r="F59" s="9"/>
-      <c r="G59" s="9"/>
-      <c r="H59" s="9" t="s">
+      <c r="C59" s="8" t="s">
+        <v>37</v>
+      </c>
+      <c r="D59" s="8"/>
+      <c r="E59" s="8"/>
+      <c r="F59" s="8"/>
+      <c r="G59" s="8"/>
+      <c r="H59" s="8" t="s">
         <v>110</v>
       </c>
     </row>
@@ -2272,230 +2288,230 @@
       <c r="H60" s="12"/>
     </row>
     <row r="61" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A61" s="11" t="s">
+      <c r="A61" s="10" t="s">
         <v>115</v>
       </c>
-      <c r="B61" s="11"/>
-      <c r="C61" s="11"/>
-      <c r="D61" s="11"/>
-      <c r="E61" s="11"/>
-      <c r="F61" s="11"/>
-      <c r="G61" s="11"/>
-      <c r="H61" s="11"/>
+      <c r="B61" s="10"/>
+      <c r="C61" s="10"/>
+      <c r="D61" s="10"/>
+      <c r="E61" s="10"/>
+      <c r="F61" s="10"/>
+      <c r="G61" s="10"/>
+      <c r="H61" s="10"/>
     </row>
     <row r="62" spans="1:8" ht="43.5" x14ac:dyDescent="0.35">
-      <c r="A62" s="9"/>
-      <c r="B62" s="9" t="s">
+      <c r="A62" s="8"/>
+      <c r="B62" s="8" t="s">
         <v>116</v>
       </c>
-      <c r="C62" s="9" t="s">
-        <v>37</v>
-      </c>
-      <c r="D62" s="9"/>
-      <c r="E62" s="9">
+      <c r="C62" s="8" t="s">
+        <v>37</v>
+      </c>
+      <c r="D62" s="8"/>
+      <c r="E62" s="8">
         <v>12</v>
       </c>
-      <c r="F62" s="9" t="s">
-        <v>37</v>
-      </c>
-      <c r="G62" s="9"/>
-      <c r="H62" s="9" t="s">
+      <c r="F62" s="8" t="s">
+        <v>37</v>
+      </c>
+      <c r="G62" s="8"/>
+      <c r="H62" s="8" t="s">
         <v>110</v>
       </c>
     </row>
     <row r="63" spans="1:8" ht="29" x14ac:dyDescent="0.35">
-      <c r="A63" s="9"/>
-      <c r="B63" s="9" t="s">
+      <c r="A63" s="8"/>
+      <c r="B63" s="8" t="s">
         <v>117</v>
       </c>
-      <c r="C63" s="9" t="s">
-        <v>37</v>
-      </c>
-      <c r="D63" s="9"/>
-      <c r="E63" s="9">
+      <c r="C63" s="8" t="s">
+        <v>37</v>
+      </c>
+      <c r="D63" s="8"/>
+      <c r="E63" s="8">
         <v>9</v>
       </c>
-      <c r="F63" s="9" t="s">
-        <v>37</v>
-      </c>
-      <c r="G63" s="9"/>
-      <c r="H63" s="9" t="s">
+      <c r="F63" s="8" t="s">
+        <v>37</v>
+      </c>
+      <c r="G63" s="8"/>
+      <c r="H63" s="8" t="s">
         <v>110</v>
       </c>
     </row>
     <row r="64" spans="1:8" ht="29" x14ac:dyDescent="0.35">
-      <c r="A64" s="9"/>
-      <c r="B64" s="9" t="s">
+      <c r="A64" s="8"/>
+      <c r="B64" s="8" t="s">
         <v>118</v>
       </c>
-      <c r="C64" s="9" t="s">
-        <v>37</v>
-      </c>
-      <c r="D64" s="9"/>
-      <c r="E64" s="9">
+      <c r="C64" s="8" t="s">
+        <v>37</v>
+      </c>
+      <c r="D64" s="8"/>
+      <c r="E64" s="8">
         <v>3</v>
       </c>
-      <c r="F64" s="9" t="s">
-        <v>37</v>
-      </c>
-      <c r="G64" s="9"/>
-      <c r="H64" s="9" t="s">
+      <c r="F64" s="8" t="s">
+        <v>37</v>
+      </c>
+      <c r="G64" s="8"/>
+      <c r="H64" s="8" t="s">
         <v>110</v>
       </c>
     </row>
     <row r="65" spans="1:8" ht="29" x14ac:dyDescent="0.35">
-      <c r="A65" s="9"/>
-      <c r="B65" s="9" t="s">
+      <c r="A65" s="8"/>
+      <c r="B65" s="8" t="s">
         <v>48</v>
       </c>
-      <c r="C65" s="9" t="s">
-        <v>37</v>
-      </c>
-      <c r="D65" s="9"/>
-      <c r="E65" s="9"/>
-      <c r="F65" s="9"/>
-      <c r="G65" s="9"/>
-      <c r="H65" s="9" t="s">
+      <c r="C65" s="8" t="s">
+        <v>37</v>
+      </c>
+      <c r="D65" s="8"/>
+      <c r="E65" s="8"/>
+      <c r="F65" s="8"/>
+      <c r="G65" s="8"/>
+      <c r="H65" s="8" t="s">
         <v>110</v>
       </c>
     </row>
     <row r="66" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A66" s="11" t="s">
+      <c r="A66" s="10" t="s">
         <v>119</v>
       </c>
-      <c r="B66" s="11"/>
-      <c r="C66" s="11"/>
-      <c r="D66" s="11"/>
-      <c r="E66" s="11"/>
-      <c r="F66" s="11"/>
-      <c r="G66" s="11"/>
-      <c r="H66" s="11"/>
+      <c r="B66" s="10"/>
+      <c r="C66" s="10"/>
+      <c r="D66" s="10"/>
+      <c r="E66" s="10"/>
+      <c r="F66" s="10"/>
+      <c r="G66" s="10"/>
+      <c r="H66" s="10"/>
     </row>
     <row r="67" spans="1:8" ht="145" x14ac:dyDescent="0.35">
-      <c r="A67" s="9"/>
-      <c r="B67" s="9" t="s">
+      <c r="A67" s="8"/>
+      <c r="B67" s="8" t="s">
         <v>120</v>
       </c>
-      <c r="C67" s="9" t="s">
-        <v>37</v>
-      </c>
-      <c r="D67" s="9"/>
-      <c r="E67" s="9">
+      <c r="C67" s="8" t="s">
+        <v>37</v>
+      </c>
+      <c r="D67" s="8"/>
+      <c r="E67" s="8">
         <v>17</v>
       </c>
-      <c r="F67" s="9" t="s">
-        <v>37</v>
-      </c>
-      <c r="G67" s="9" t="s">
+      <c r="F67" s="8" t="s">
+        <v>37</v>
+      </c>
+      <c r="G67" s="8" t="s">
         <v>121</v>
       </c>
-      <c r="H67" s="9" t="s">
+      <c r="H67" s="8" t="s">
         <v>110</v>
       </c>
     </row>
     <row r="68" spans="1:8" ht="145" x14ac:dyDescent="0.35">
-      <c r="A68" s="9"/>
-      <c r="B68" s="9" t="s">
+      <c r="A68" s="8"/>
+      <c r="B68" s="8" t="s">
         <v>122</v>
       </c>
-      <c r="C68" s="9" t="s">
-        <v>37</v>
-      </c>
-      <c r="D68" s="9" t="s">
+      <c r="C68" s="8" t="s">
+        <v>37</v>
+      </c>
+      <c r="D68" s="8" t="s">
         <v>123</v>
       </c>
-      <c r="E68" s="9">
+      <c r="E68" s="8">
         <v>13</v>
       </c>
-      <c r="F68" s="9" t="s">
-        <v>37</v>
-      </c>
-      <c r="G68" s="9" t="s">
+      <c r="F68" s="8" t="s">
+        <v>37</v>
+      </c>
+      <c r="G68" s="8" t="s">
         <v>124</v>
       </c>
-      <c r="H68" s="9" t="s">
+      <c r="H68" s="8" t="s">
         <v>110</v>
       </c>
     </row>
     <row r="69" spans="1:8" ht="145" x14ac:dyDescent="0.35">
-      <c r="A69" s="9"/>
-      <c r="B69" s="9" t="s">
+      <c r="A69" s="8"/>
+      <c r="B69" s="8" t="s">
         <v>125</v>
       </c>
-      <c r="C69" s="9" t="s">
-        <v>37</v>
-      </c>
-      <c r="D69" s="9" t="s">
+      <c r="C69" s="8" t="s">
+        <v>37</v>
+      </c>
+      <c r="D69" s="8" t="s">
         <v>123</v>
       </c>
-      <c r="E69" s="9">
+      <c r="E69" s="8">
         <v>8</v>
       </c>
-      <c r="F69" s="9" t="s">
-        <v>37</v>
-      </c>
-      <c r="G69" s="9" t="s">
+      <c r="F69" s="8" t="s">
+        <v>37</v>
+      </c>
+      <c r="G69" s="8" t="s">
         <v>126</v>
       </c>
-      <c r="H69" s="9" t="s">
+      <c r="H69" s="8" t="s">
         <v>110</v>
       </c>
     </row>
     <row r="70" spans="1:8" ht="87" x14ac:dyDescent="0.35">
-      <c r="A70" s="9"/>
-      <c r="B70" s="9" t="s">
+      <c r="A70" s="8"/>
+      <c r="B70" s="8" t="s">
         <v>127</v>
       </c>
-      <c r="C70" s="9" t="s">
-        <v>37</v>
-      </c>
-      <c r="D70" s="9" t="s">
+      <c r="C70" s="8" t="s">
+        <v>37</v>
+      </c>
+      <c r="D70" s="8" t="s">
         <v>123</v>
       </c>
-      <c r="E70" s="9">
+      <c r="E70" s="8">
         <v>6</v>
       </c>
-      <c r="F70" s="9" t="s">
-        <v>37</v>
-      </c>
-      <c r="G70" s="9"/>
-      <c r="H70" s="9" t="s">
+      <c r="F70" s="8" t="s">
+        <v>37</v>
+      </c>
+      <c r="G70" s="8"/>
+      <c r="H70" s="8" t="s">
         <v>110</v>
       </c>
     </row>
     <row r="71" spans="1:8" ht="87" x14ac:dyDescent="0.35">
-      <c r="A71" s="9"/>
-      <c r="B71" s="9" t="s">
+      <c r="A71" s="8"/>
+      <c r="B71" s="8" t="s">
         <v>128</v>
       </c>
-      <c r="C71" s="9" t="s">
-        <v>37</v>
-      </c>
-      <c r="D71" s="9" t="s">
+      <c r="C71" s="8" t="s">
+        <v>37</v>
+      </c>
+      <c r="D71" s="8" t="s">
         <v>123</v>
       </c>
-      <c r="E71" s="9"/>
-      <c r="F71" s="9"/>
-      <c r="G71" s="9" t="s">
+      <c r="E71" s="8"/>
+      <c r="F71" s="8"/>
+      <c r="G71" s="8" t="s">
         <v>67</v>
       </c>
-      <c r="H71" s="9" t="s">
+      <c r="H71" s="8" t="s">
         <v>110</v>
       </c>
     </row>
     <row r="72" spans="1:8" ht="29" x14ac:dyDescent="0.35">
-      <c r="A72" s="9"/>
-      <c r="B72" s="9" t="s">
+      <c r="A72" s="8"/>
+      <c r="B72" s="8" t="s">
         <v>48</v>
       </c>
-      <c r="C72" s="9" t="s">
-        <v>37</v>
-      </c>
-      <c r="D72" s="9"/>
-      <c r="E72" s="9"/>
-      <c r="F72" s="9"/>
-      <c r="G72" s="9"/>
-      <c r="H72" s="9" t="s">
+      <c r="C72" s="8" t="s">
+        <v>37</v>
+      </c>
+      <c r="D72" s="8"/>
+      <c r="E72" s="8"/>
+      <c r="F72" s="8"/>
+      <c r="G72" s="8"/>
+      <c r="H72" s="8" t="s">
         <v>110</v>
       </c>
     </row>
@@ -2512,268 +2528,268 @@
       <c r="H73" s="12"/>
     </row>
     <row r="74" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A74" s="11" t="s">
+      <c r="A74" s="10" t="s">
         <v>130</v>
       </c>
-      <c r="B74" s="11"/>
-      <c r="C74" s="11"/>
-      <c r="D74" s="11"/>
-      <c r="E74" s="11"/>
-      <c r="F74" s="11"/>
-      <c r="G74" s="11"/>
-      <c r="H74" s="11"/>
+      <c r="B74" s="10"/>
+      <c r="C74" s="10"/>
+      <c r="D74" s="10"/>
+      <c r="E74" s="10"/>
+      <c r="F74" s="10"/>
+      <c r="G74" s="10"/>
+      <c r="H74" s="10"/>
     </row>
     <row r="75" spans="1:8" ht="101.5" x14ac:dyDescent="0.35">
-      <c r="A75" s="9"/>
-      <c r="B75" s="9" t="s">
+      <c r="A75" s="8"/>
+      <c r="B75" s="8" t="s">
         <v>131</v>
       </c>
-      <c r="C75" s="9" t="s">
-        <v>37</v>
-      </c>
-      <c r="D75" s="9" t="s">
+      <c r="C75" s="8" t="s">
+        <v>37</v>
+      </c>
+      <c r="D75" s="8" t="s">
         <v>132</v>
       </c>
-      <c r="E75" s="9">
+      <c r="E75" s="8">
         <v>7</v>
       </c>
-      <c r="F75" s="9" t="s">
-        <v>37</v>
-      </c>
-      <c r="G75" s="9"/>
-      <c r="H75" s="9" t="s">
+      <c r="F75" s="8" t="s">
+        <v>37</v>
+      </c>
+      <c r="G75" s="8"/>
+      <c r="H75" s="8" t="s">
         <v>133</v>
       </c>
     </row>
     <row r="76" spans="1:8" ht="116" x14ac:dyDescent="0.35">
-      <c r="A76" s="9"/>
-      <c r="B76" s="9" t="s">
+      <c r="A76" s="8"/>
+      <c r="B76" s="8" t="s">
         <v>134</v>
       </c>
-      <c r="C76" s="9" t="s">
-        <v>37</v>
-      </c>
-      <c r="D76" s="9" t="s">
+      <c r="C76" s="8" t="s">
+        <v>37</v>
+      </c>
+      <c r="D76" s="8" t="s">
         <v>135</v>
       </c>
-      <c r="E76" s="9">
+      <c r="E76" s="8">
         <v>3</v>
       </c>
-      <c r="F76" s="9" t="s">
-        <v>37</v>
-      </c>
-      <c r="G76" s="9"/>
-      <c r="H76" s="9" t="s">
+      <c r="F76" s="8" t="s">
+        <v>37</v>
+      </c>
+      <c r="G76" s="8"/>
+      <c r="H76" s="8" t="s">
         <v>133</v>
       </c>
     </row>
     <row r="77" spans="1:8" ht="116" x14ac:dyDescent="0.35">
-      <c r="A77" s="9"/>
-      <c r="B77" s="9" t="s">
+      <c r="A77" s="8"/>
+      <c r="B77" s="8" t="s">
         <v>136</v>
       </c>
-      <c r="C77" s="9" t="s">
-        <v>37</v>
-      </c>
-      <c r="D77" s="9" t="s">
+      <c r="C77" s="8" t="s">
+        <v>37</v>
+      </c>
+      <c r="D77" s="8" t="s">
         <v>135</v>
       </c>
-      <c r="E77" s="9">
+      <c r="E77" s="8">
         <v>2</v>
       </c>
-      <c r="F77" s="9" t="s">
-        <v>37</v>
-      </c>
-      <c r="G77" s="9"/>
-      <c r="H77" s="9" t="s">
+      <c r="F77" s="8" t="s">
+        <v>37</v>
+      </c>
+      <c r="G77" s="8"/>
+      <c r="H77" s="8" t="s">
         <v>133</v>
       </c>
     </row>
     <row r="78" spans="1:8" ht="116" x14ac:dyDescent="0.35">
-      <c r="A78" s="9"/>
-      <c r="B78" s="9" t="s">
+      <c r="A78" s="8"/>
+      <c r="B78" s="8" t="s">
         <v>137</v>
       </c>
-      <c r="C78" s="9" t="s">
-        <v>37</v>
-      </c>
-      <c r="D78" s="9" t="s">
+      <c r="C78" s="8" t="s">
+        <v>37</v>
+      </c>
+      <c r="D78" s="8" t="s">
         <v>135</v>
       </c>
-      <c r="E78" s="9">
+      <c r="E78" s="8">
         <v>3</v>
       </c>
-      <c r="F78" s="9" t="s">
-        <v>37</v>
-      </c>
-      <c r="G78" s="9"/>
-      <c r="H78" s="9" t="s">
+      <c r="F78" s="8" t="s">
+        <v>37</v>
+      </c>
+      <c r="G78" s="8"/>
+      <c r="H78" s="8" t="s">
         <v>133</v>
       </c>
     </row>
     <row r="79" spans="1:8" ht="58" x14ac:dyDescent="0.35">
-      <c r="A79" s="9"/>
-      <c r="B79" s="9" t="s">
+      <c r="A79" s="8"/>
+      <c r="B79" s="8" t="s">
         <v>138</v>
       </c>
-      <c r="C79" s="9" t="s">
-        <v>37</v>
-      </c>
-      <c r="D79" s="9" t="s">
+      <c r="C79" s="8" t="s">
+        <v>37</v>
+      </c>
+      <c r="D79" s="8" t="s">
         <v>139</v>
       </c>
-      <c r="E79" s="9">
+      <c r="E79" s="8">
         <v>5</v>
       </c>
-      <c r="F79" s="9" t="s">
-        <v>37</v>
-      </c>
-      <c r="G79" s="9"/>
-      <c r="H79" s="9" t="s">
+      <c r="F79" s="8" t="s">
+        <v>37</v>
+      </c>
+      <c r="G79" s="8"/>
+      <c r="H79" s="8" t="s">
         <v>133</v>
       </c>
     </row>
     <row r="80" spans="1:8" ht="29" x14ac:dyDescent="0.35">
-      <c r="A80" s="9"/>
-      <c r="B80" s="9" t="s">
+      <c r="A80" s="8"/>
+      <c r="B80" s="8" t="s">
         <v>48</v>
       </c>
-      <c r="C80" s="9" t="s">
-        <v>37</v>
-      </c>
-      <c r="D80" s="9"/>
-      <c r="E80" s="9"/>
-      <c r="F80" s="9"/>
-      <c r="G80" s="9"/>
-      <c r="H80" s="9" t="s">
+      <c r="C80" s="8" t="s">
+        <v>37</v>
+      </c>
+      <c r="D80" s="8"/>
+      <c r="E80" s="8"/>
+      <c r="F80" s="8"/>
+      <c r="G80" s="8"/>
+      <c r="H80" s="8" t="s">
         <v>133</v>
       </c>
     </row>
     <row r="81" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A81" s="11" t="s">
+      <c r="A81" s="10" t="s">
         <v>140</v>
       </c>
-      <c r="B81" s="11"/>
-      <c r="C81" s="11"/>
-      <c r="D81" s="11"/>
-      <c r="E81" s="11"/>
-      <c r="F81" s="11"/>
-      <c r="G81" s="11"/>
-      <c r="H81" s="11"/>
+      <c r="B81" s="10"/>
+      <c r="C81" s="10"/>
+      <c r="D81" s="10"/>
+      <c r="E81" s="10"/>
+      <c r="F81" s="10"/>
+      <c r="G81" s="10"/>
+      <c r="H81" s="10"/>
     </row>
     <row r="82" spans="1:8" ht="87" x14ac:dyDescent="0.35">
-      <c r="A82" s="9"/>
-      <c r="B82" s="9" t="s">
+      <c r="A82" s="8"/>
+      <c r="B82" s="8" t="s">
         <v>141</v>
       </c>
-      <c r="C82" s="9" t="s">
+      <c r="C82" s="8" t="s">
         <v>142</v>
       </c>
-      <c r="D82" s="9" t="s">
+      <c r="D82" s="8" t="s">
         <v>143</v>
       </c>
-      <c r="E82" s="9"/>
-      <c r="F82" s="9" t="s">
+      <c r="E82" s="8"/>
+      <c r="F82" s="8" t="s">
         <v>142</v>
       </c>
-      <c r="G82" s="9" t="s">
+      <c r="G82" s="8" t="s">
         <v>144</v>
       </c>
-      <c r="H82" s="9"/>
+      <c r="H82" s="8"/>
     </row>
     <row r="83" spans="1:8" ht="72.5" x14ac:dyDescent="0.35">
-      <c r="A83" s="9"/>
-      <c r="B83" s="9" t="s">
+      <c r="A83" s="8"/>
+      <c r="B83" s="8" t="s">
         <v>145</v>
       </c>
-      <c r="C83" s="9" t="s">
+      <c r="C83" s="8" t="s">
         <v>146</v>
       </c>
-      <c r="D83" s="9" t="s">
+      <c r="D83" s="8" t="s">
         <v>147</v>
       </c>
-      <c r="E83" s="9"/>
-      <c r="F83" s="9" t="s">
+      <c r="E83" s="8"/>
+      <c r="F83" s="8" t="s">
         <v>146</v>
       </c>
-      <c r="G83" s="9" t="s">
+      <c r="G83" s="8" t="s">
         <v>148</v>
       </c>
-      <c r="H83" s="9"/>
+      <c r="H83" s="8"/>
     </row>
     <row r="84" spans="1:8" ht="72.5" x14ac:dyDescent="0.35">
-      <c r="A84" s="9"/>
-      <c r="B84" s="9" t="s">
+      <c r="A84" s="8"/>
+      <c r="B84" s="8" t="s">
         <v>149</v>
       </c>
-      <c r="C84" s="9" t="s">
+      <c r="C84" s="8" t="s">
         <v>142</v>
       </c>
-      <c r="D84" s="9" t="s">
+      <c r="D84" s="8" t="s">
         <v>150</v>
       </c>
-      <c r="E84" s="9"/>
-      <c r="F84" s="9" t="s">
+      <c r="E84" s="8"/>
+      <c r="F84" s="8" t="s">
         <v>142</v>
       </c>
-      <c r="G84" s="9" t="s">
+      <c r="G84" s="8" t="s">
         <v>151</v>
       </c>
-      <c r="H84" s="9"/>
+      <c r="H84" s="8"/>
     </row>
     <row r="85" spans="1:8" ht="29" x14ac:dyDescent="0.35">
-      <c r="A85" s="9"/>
-      <c r="B85" s="9" t="s">
+      <c r="A85" s="8"/>
+      <c r="B85" s="8" t="s">
         <v>152</v>
       </c>
-      <c r="C85" s="9" t="s">
-        <v>37</v>
-      </c>
-      <c r="D85" s="9"/>
-      <c r="E85" s="9">
+      <c r="C85" s="8" t="s">
+        <v>37</v>
+      </c>
+      <c r="D85" s="8"/>
+      <c r="E85" s="8">
         <v>6</v>
       </c>
-      <c r="F85" s="9" t="s">
-        <v>37</v>
-      </c>
-      <c r="G85" s="9"/>
-      <c r="H85" s="9" t="s">
+      <c r="F85" s="8" t="s">
+        <v>37</v>
+      </c>
+      <c r="G85" s="8"/>
+      <c r="H85" s="8" t="s">
         <v>133</v>
       </c>
     </row>
     <row r="86" spans="1:8" ht="43.5" x14ac:dyDescent="0.35">
-      <c r="A86" s="9"/>
-      <c r="B86" s="9" t="s">
+      <c r="A86" s="8"/>
+      <c r="B86" s="8" t="s">
         <v>153</v>
       </c>
-      <c r="C86" s="9" t="s">
-        <v>37</v>
-      </c>
-      <c r="D86" s="9"/>
-      <c r="E86" s="9">
+      <c r="C86" s="8" t="s">
+        <v>37</v>
+      </c>
+      <c r="D86" s="8"/>
+      <c r="E86" s="8">
         <v>5</v>
       </c>
-      <c r="F86" s="9" t="s">
-        <v>37</v>
-      </c>
-      <c r="G86" s="9"/>
-      <c r="H86" s="9" t="s">
+      <c r="F86" s="8" t="s">
+        <v>37</v>
+      </c>
+      <c r="G86" s="8"/>
+      <c r="H86" s="8" t="s">
         <v>133</v>
       </c>
     </row>
     <row r="87" spans="1:8" ht="29" x14ac:dyDescent="0.35">
-      <c r="A87" s="9"/>
-      <c r="B87" s="9" t="s">
+      <c r="A87" s="8"/>
+      <c r="B87" s="8" t="s">
         <v>48</v>
       </c>
-      <c r="C87" s="9" t="s">
-        <v>37</v>
-      </c>
-      <c r="D87" s="9"/>
-      <c r="E87" s="9"/>
-      <c r="F87" s="9"/>
-      <c r="G87" s="9"/>
-      <c r="H87" s="9" t="s">
+      <c r="C87" s="8" t="s">
+        <v>37</v>
+      </c>
+      <c r="D87" s="8"/>
+      <c r="E87" s="8"/>
+      <c r="F87" s="8"/>
+      <c r="G87" s="8"/>
+      <c r="H87" s="8" t="s">
         <v>133</v>
       </c>
     </row>
@@ -2790,23 +2806,23 @@
       <c r="H88" s="12"/>
     </row>
     <row r="89" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A89" s="11" t="s">
+      <c r="A89" s="10" t="s">
         <v>155</v>
       </c>
-      <c r="B89" s="11"/>
-      <c r="C89" s="11"/>
-      <c r="D89" s="11"/>
-      <c r="E89" s="11"/>
-      <c r="F89" s="11"/>
-      <c r="G89" s="11"/>
-      <c r="H89" s="11"/>
+      <c r="B89" s="10"/>
+      <c r="C89" s="10"/>
+      <c r="D89" s="10"/>
+      <c r="E89" s="10"/>
+      <c r="F89" s="10"/>
+      <c r="G89" s="10"/>
+      <c r="H89" s="10"/>
     </row>
     <row r="90" spans="1:8" ht="174" x14ac:dyDescent="0.35">
-      <c r="A90" s="9"/>
+      <c r="A90" s="8"/>
       <c r="B90" t="s">
         <v>156</v>
       </c>
-      <c r="C90" s="9" t="s">
+      <c r="C90" s="8" t="s">
         <v>157</v>
       </c>
       <c r="E90">
@@ -2815,7 +2831,7 @@
       <c r="F90" t="s">
         <v>37</v>
       </c>
-      <c r="G90" s="9" t="s">
+      <c r="G90" s="8" t="s">
         <v>158</v>
       </c>
       <c r="H90" t="s">
@@ -2823,14 +2839,14 @@
       </c>
     </row>
     <row r="91" spans="1:8" ht="116" x14ac:dyDescent="0.35">
-      <c r="A91" s="9"/>
+      <c r="A91" s="8"/>
       <c r="B91" t="s">
         <v>159</v>
       </c>
-      <c r="C91" s="9" t="s">
+      <c r="C91" s="8" t="s">
         <v>160</v>
       </c>
-      <c r="D91" s="9" t="s">
+      <c r="D91" s="8" t="s">
         <v>161</v>
       </c>
       <c r="E91">
@@ -2844,11 +2860,11 @@
       </c>
     </row>
     <row r="92" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A92" s="9"/>
+      <c r="A92" s="8"/>
       <c r="B92" t="s">
         <v>162</v>
       </c>
-      <c r="C92" s="9" t="s">
+      <c r="C92" s="8" t="s">
         <v>37</v>
       </c>
       <c r="E92">
@@ -2862,131 +2878,131 @@
       </c>
     </row>
     <row r="93" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A93" s="9"/>
+      <c r="A93" s="8"/>
       <c r="B93" t="s">
         <v>48</v>
       </c>
-      <c r="C93" s="9" t="s">
+      <c r="C93" s="8" t="s">
         <v>37</v>
       </c>
     </row>
     <row r="94" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A94" s="11" t="s">
+      <c r="A94" s="10" t="s">
         <v>163</v>
       </c>
-      <c r="B94" s="11"/>
-      <c r="C94" s="11"/>
-      <c r="D94" s="11"/>
-      <c r="E94" s="11"/>
-      <c r="F94" s="11"/>
-      <c r="G94" s="11"/>
-      <c r="H94" s="11"/>
+      <c r="B94" s="10"/>
+      <c r="C94" s="10"/>
+      <c r="D94" s="10"/>
+      <c r="E94" s="10"/>
+      <c r="F94" s="10"/>
+      <c r="G94" s="10"/>
+      <c r="H94" s="10"/>
     </row>
     <row r="95" spans="1:8" ht="43.5" x14ac:dyDescent="0.35">
-      <c r="A95" s="9"/>
-      <c r="B95" s="9" t="s">
+      <c r="A95" s="8"/>
+      <c r="B95" s="8" t="s">
         <v>164</v>
       </c>
-      <c r="C95" s="9" t="s">
-        <v>37</v>
-      </c>
-      <c r="D95" s="9"/>
-      <c r="E95" s="9"/>
-      <c r="F95" s="9"/>
-      <c r="G95" s="9" t="s">
+      <c r="C95" s="8" t="s">
+        <v>37</v>
+      </c>
+      <c r="D95" s="8"/>
+      <c r="E95" s="8"/>
+      <c r="F95" s="8"/>
+      <c r="G95" s="8" t="s">
         <v>67</v>
       </c>
-      <c r="H95" s="9" t="s">
+      <c r="H95" s="8" t="s">
         <v>165</v>
       </c>
     </row>
     <row r="96" spans="1:8" ht="29" x14ac:dyDescent="0.35">
-      <c r="A96" s="9"/>
-      <c r="B96" s="9" t="s">
+      <c r="A96" s="8"/>
+      <c r="B96" s="8" t="s">
         <v>166</v>
       </c>
-      <c r="C96" s="9" t="s">
-        <v>37</v>
-      </c>
-      <c r="D96" s="9"/>
-      <c r="E96" s="9"/>
-      <c r="F96" s="9">
+      <c r="C96" s="8" t="s">
+        <v>37</v>
+      </c>
+      <c r="D96" s="8"/>
+      <c r="E96" s="8"/>
+      <c r="F96" s="8">
         <v>3</v>
       </c>
-      <c r="G96" s="9"/>
-      <c r="H96" s="9" t="s">
+      <c r="G96" s="8"/>
+      <c r="H96" s="8" t="s">
         <v>165</v>
       </c>
     </row>
     <row r="97" spans="1:8" ht="101.5" x14ac:dyDescent="0.35">
-      <c r="A97" s="9"/>
-      <c r="B97" s="9" t="s">
+      <c r="A97" s="8"/>
+      <c r="B97" s="8" t="s">
         <v>167</v>
       </c>
-      <c r="C97" s="9" t="s">
-        <v>37</v>
-      </c>
-      <c r="D97" s="9" t="s">
+      <c r="C97" s="8" t="s">
+        <v>37</v>
+      </c>
+      <c r="D97" s="8" t="s">
         <v>168</v>
       </c>
-      <c r="E97" s="9"/>
-      <c r="F97" s="9">
+      <c r="E97" s="8"/>
+      <c r="F97" s="8">
         <v>4</v>
       </c>
-      <c r="G97" s="9"/>
-      <c r="H97" s="9" t="s">
+      <c r="G97" s="8"/>
+      <c r="H97" s="8" t="s">
         <v>165</v>
       </c>
     </row>
     <row r="98" spans="1:8" ht="43.5" x14ac:dyDescent="0.35">
-      <c r="A98" s="9"/>
-      <c r="B98" s="9" t="s">
+      <c r="A98" s="8"/>
+      <c r="B98" s="8" t="s">
         <v>169</v>
       </c>
-      <c r="C98" s="9" t="s">
-        <v>37</v>
-      </c>
-      <c r="D98" s="9"/>
-      <c r="E98" s="9"/>
-      <c r="F98" s="9">
+      <c r="C98" s="8" t="s">
+        <v>37</v>
+      </c>
+      <c r="D98" s="8"/>
+      <c r="E98" s="8"/>
+      <c r="F98" s="8">
         <v>5</v>
       </c>
-      <c r="G98" s="9"/>
-      <c r="H98" s="9" t="s">
+      <c r="G98" s="8"/>
+      <c r="H98" s="8" t="s">
         <v>165</v>
       </c>
     </row>
     <row r="99" spans="1:8" ht="43.5" x14ac:dyDescent="0.35">
-      <c r="A99" s="9"/>
-      <c r="B99" s="9" t="s">
+      <c r="A99" s="8"/>
+      <c r="B99" s="8" t="s">
         <v>170</v>
       </c>
-      <c r="C99" s="9" t="s">
-        <v>37</v>
-      </c>
-      <c r="D99" s="9"/>
-      <c r="E99" s="9"/>
-      <c r="F99" s="9">
+      <c r="C99" s="8" t="s">
+        <v>37</v>
+      </c>
+      <c r="D99" s="8"/>
+      <c r="E99" s="8"/>
+      <c r="F99" s="8">
         <v>8</v>
       </c>
-      <c r="G99" s="9"/>
-      <c r="H99" s="9" t="s">
+      <c r="G99" s="8"/>
+      <c r="H99" s="8" t="s">
         <v>165</v>
       </c>
     </row>
     <row r="100" spans="1:8" ht="29" x14ac:dyDescent="0.35">
-      <c r="A100" s="9"/>
-      <c r="B100" s="9" t="s">
+      <c r="A100" s="8"/>
+      <c r="B100" s="8" t="s">
         <v>48</v>
       </c>
-      <c r="C100" s="9" t="s">
-        <v>37</v>
-      </c>
-      <c r="D100" s="9"/>
-      <c r="E100" s="9"/>
-      <c r="F100" s="9"/>
-      <c r="G100" s="9"/>
-      <c r="H100" s="9" t="s">
+      <c r="C100" s="8" t="s">
+        <v>37</v>
+      </c>
+      <c r="D100" s="8"/>
+      <c r="E100" s="8"/>
+      <c r="F100" s="8"/>
+      <c r="G100" s="8"/>
+      <c r="H100" s="8" t="s">
         <v>165</v>
       </c>
     </row>
@@ -3001,12 +3017,12 @@
     <mergeCell ref="A73:H73"/>
     <mergeCell ref="A74:H74"/>
     <mergeCell ref="A81:H81"/>
+    <mergeCell ref="A54:H54"/>
     <mergeCell ref="B1:J1"/>
     <mergeCell ref="B2:J2"/>
     <mergeCell ref="A44:H44"/>
     <mergeCell ref="A48:H48"/>
     <mergeCell ref="A49:H49"/>
-    <mergeCell ref="A54:H54"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -3014,18 +3030,30 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{26BBF184-5DF4-4140-BC06-EDE079C5024C}">
-  <dimension ref="A1"/>
+  <dimension ref="B5"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
-  <sheetData/>
+  <sheetData>
+    <row r="5" spans="2:2" x14ac:dyDescent="0.35">
+      <c r="B5" t="s">
+        <v>141</v>
+      </c>
+    </row>
+  </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DE062A2B-7814-4D62-BFF1-4EDA02A4C168}">
-  <dimension ref="A1"/>
+  <dimension ref="B8"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
-  <sheetData/>
+  <sheetData>
+    <row r="8" spans="2:2" x14ac:dyDescent="0.35">
+      <c r="B8" t="s">
+        <v>141</v>
+      </c>
+    </row>
+  </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>